<commit_message>
Deferred-items pass: redirect pinning (P2-21), amount/wallet validation (DI-2/SEC-2), discharge guards (BIZ-5/6), reject state (WF1-1), 60s sync cache (SYNC-1), PII encryption (SEC-3), mailer hooks (NOTIF-1/2), live category filters (P1-13), dead links fixed (P1-12/P2-18), stale files archived (P2-20), sitemap (P3-22), README refresh (P3-25)
</commit_message>
<xml_diff>
--- a/audits/20260802/reports/master-audit-20260802.xlsx
+++ b/audits/20260802/reports/master-audit-20260802.xlsx
@@ -1150,7 +1150,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -2866,7 +2866,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -2918,7 +2918,7 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -3750,7 +3750,7 @@
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -4010,7 +4010,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -4374,7 +4374,7 @@
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
@@ -4426,7 +4426,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">

</xml_diff>